<commit_message>
Update board.xlsx from Google Sheets
</commit_message>
<xml_diff>
--- a/data/board.xlsx
+++ b/data/board.xlsx
@@ -9,14 +9,14 @@
   <calcPr/>
   <extLst>
     <ext uri="GoogleSheetsCustomDataVersion2">
-      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId5" roundtripDataChecksum="8K6PCeW4BM2XUVG+bQ3gjFmdTeBxXQ5I3cedOTzrRJQ="/>
+      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId5" roundtripDataChecksum="ubZm7D5ZblmA28W8TD2l9ksljvMNFCDpqjvqySgxPoQ="/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="15">
   <si>
     <t>플레이 날짜</t>
   </si>
@@ -33,74 +33,41 @@
     <t>감점</t>
   </si>
   <si>
-    <t>콩심기</t>
+    <t>출석 체크</t>
   </si>
   <si>
-    <t>hyoo</t>
+    <t>Julia</t>
   </si>
   <si>
-    <t>hsko</t>
+    <t>Jungmin</t>
   </si>
   <si>
-    <t>jwkim</t>
+    <t>Sophia</t>
   </si>
   <si>
-    <t>spark</t>
+    <t>Hyangyoo</t>
   </si>
   <si>
-    <t>wchoi</t>
+    <t>Jamie</t>
   </si>
   <si>
-    <t>Take 5!</t>
+    <t>Exploding Kittens</t>
   </si>
   <si>
-    <t>ryan.lim</t>
+    <t>One Night Ultimate Werewolf</t>
   </si>
   <si>
-    <t>jjung</t>
+    <t>Clue | 클루</t>
   </si>
   <si>
-    <t>jsung</t>
-  </si>
-  <si>
-    <t>타코 캣 고트 치즈 피자</t>
-  </si>
-  <si>
-    <t>schoi</t>
-  </si>
-  <si>
-    <t>cnjang</t>
-  </si>
-  <si>
-    <t>jmkim</t>
-  </si>
-  <si>
-    <t>hjkim</t>
-  </si>
-  <si>
-    <t>spjoo</t>
-  </si>
-  <si>
-    <t>mkyung</t>
-  </si>
-  <si>
-    <t>jekim</t>
-  </si>
-  <si>
-    <t>epark</t>
-  </si>
-  <si>
-    <t>sryu</t>
-  </si>
-  <si>
-    <t>루미큐브</t>
+    <t>Bohnanaza | 콩심기</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="4">
+  <fonts count="3">
     <font>
       <sz val="11.0"/>
       <color theme="1"/>
@@ -109,11 +76,6 @@
     </font>
     <font>
       <b/>
-      <sz val="11.0"/>
-      <color theme="1"/>
-      <name val="Aptos Narrow"/>
-    </font>
-    <font>
       <sz val="11.0"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
@@ -152,7 +114,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="4">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -160,18 +122,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf borderId="1" fillId="0" fontId="2" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
     <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" vertical="center"/>
-    </xf>
-    <xf borderId="1" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" vertical="center"/>
-    </xf>
-    <xf borderId="1" fillId="0" fontId="3" numFmtId="14" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
   </cellXfs>
@@ -413,16 +366,16 @@
     </row>
     <row r="2">
       <c r="A2" s="2">
-        <v>46028.0</v>
+        <v>46046.0</v>
       </c>
       <c r="B2" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C2" s="3" t="s">
         <v>6</v>
       </c>
       <c r="D2" s="3">
-        <v>3.0</v>
+        <v>2.0</v>
       </c>
       <c r="E2" s="3">
         <v>0.0</v>
@@ -430,12 +383,12 @@
     </row>
     <row r="3">
       <c r="A3" s="2">
-        <v>46028.0</v>
+        <v>46046.0</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="C3" s="3" t="s">
         <v>7</v>
       </c>
       <c r="D3" s="3">
@@ -447,16 +400,16 @@
     </row>
     <row r="4">
       <c r="A4" s="2">
-        <v>46028.0</v>
+        <v>46046.0</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="C4" s="3" t="s">
         <v>8</v>
       </c>
       <c r="D4" s="3">
-        <v>0.0</v>
+        <v>2.0</v>
       </c>
       <c r="E4" s="3">
         <v>0.0</v>
@@ -464,50 +417,50 @@
     </row>
     <row r="5">
       <c r="A5" s="2">
-        <v>46028.0</v>
+        <v>46046.0</v>
       </c>
       <c r="B5" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="C5" s="3" t="s">
         <v>9</v>
       </c>
       <c r="D5" s="3">
-        <v>0.0</v>
+        <v>2.0</v>
       </c>
       <c r="E5" s="3">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2">
-        <v>46028.0</v>
+        <v>46046.0</v>
       </c>
       <c r="B6" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="C6" s="3" t="s">
         <v>10</v>
       </c>
       <c r="D6" s="3">
-        <v>0.0</v>
+        <v>2.0</v>
       </c>
       <c r="E6" s="3">
-        <v>-1.5</v>
+        <v>0.0</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2">
-        <v>46024.0</v>
+        <v>46046.0</v>
       </c>
       <c r="B7" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="C7" s="4" t="s">
-        <v>12</v>
+      <c r="C7" s="3" t="s">
+        <v>6</v>
       </c>
       <c r="D7" s="3">
-        <v>3.0</v>
+        <v>0.0</v>
       </c>
       <c r="E7" s="3">
         <v>0.0</v>
@@ -515,16 +468,16 @@
     </row>
     <row r="8">
       <c r="A8" s="2">
-        <v>46024.0</v>
+        <v>46046.0</v>
       </c>
       <c r="B8" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="C8" s="4" t="s">
-        <v>13</v>
+      <c r="C8" s="3" t="s">
+        <v>7</v>
       </c>
       <c r="D8" s="3">
-        <v>2.0</v>
+        <v>0.0</v>
       </c>
       <c r="E8" s="3">
         <v>0.0</v>
@@ -532,12 +485,12 @@
     </row>
     <row r="9">
       <c r="A9" s="2">
-        <v>46024.0</v>
+        <v>46046.0</v>
       </c>
       <c r="B9" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="C9" s="4" t="s">
+      <c r="C9" s="3" t="s">
         <v>8</v>
       </c>
       <c r="D9" s="3">
@@ -549,50 +502,50 @@
     </row>
     <row r="10">
       <c r="A10" s="2">
-        <v>46024.0</v>
+        <v>46046.0</v>
       </c>
       <c r="B10" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="C10" s="4" t="s">
-        <v>14</v>
+      <c r="C10" s="3" t="s">
+        <v>9</v>
       </c>
       <c r="D10" s="3">
         <v>0.0</v>
       </c>
       <c r="E10" s="3">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2">
-        <v>46024.0</v>
+        <v>46046.0</v>
       </c>
       <c r="B11" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="C11" s="4" t="s">
+      <c r="C11" s="3" t="s">
         <v>10</v>
       </c>
       <c r="D11" s="3">
-        <v>0.0</v>
+        <v>3.0</v>
       </c>
       <c r="E11" s="3">
-        <v>-1.5</v>
+        <v>0.0</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2">
-        <v>46029.0</v>
+        <v>46046.0</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="C12" s="4" t="s">
-        <v>16</v>
+        <v>12</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>6</v>
       </c>
       <c r="D12" s="3">
-        <v>3.0</v>
+        <v>0.0</v>
       </c>
       <c r="E12" s="3">
         <v>0.0</v>
@@ -600,16 +553,16 @@
     </row>
     <row r="13">
       <c r="A13" s="2">
-        <v>46029.0</v>
+        <v>46046.0</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="C13" s="4" t="s">
-        <v>17</v>
+        <v>12</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>7</v>
       </c>
       <c r="D13" s="3">
-        <v>2.0</v>
+        <v>0.0</v>
       </c>
       <c r="E13" s="3">
         <v>0.0</v>
@@ -617,16 +570,16 @@
     </row>
     <row r="14">
       <c r="A14" s="2">
-        <v>46029.0</v>
+        <v>46046.0</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="C14" s="4" t="s">
-        <v>18</v>
+        <v>12</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>8</v>
       </c>
       <c r="D14" s="3">
-        <v>0.0</v>
+        <v>1.0</v>
       </c>
       <c r="E14" s="3">
         <v>0.0</v>
@@ -634,667 +587,235 @@
     </row>
     <row r="15">
       <c r="A15" s="2">
-        <v>46029.0</v>
+        <v>46046.0</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="C15" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="C15" s="3" t="s">
         <v>9</v>
       </c>
       <c r="D15" s="3">
-        <v>0.0</v>
+        <v>1.0</v>
       </c>
       <c r="E15" s="3">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2">
-        <v>46029.0</v>
+        <v>46046.0</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="C16" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="C16" s="3" t="s">
         <v>10</v>
       </c>
       <c r="D16" s="3">
-        <v>0.0</v>
+        <v>1.0</v>
       </c>
       <c r="E16" s="3">
-        <v>-1.5</v>
+        <v>0.0</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2">
-        <v>46055.0</v>
+        <v>46046.0</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="C17" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="D17" s="5">
-        <v>3.0</v>
-      </c>
-      <c r="E17" s="5">
+        <v>13</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="D17" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="E17" s="3">
         <v>0.0</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2">
-        <v>46055.0</v>
+        <v>46046.0</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="C18" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D18" s="5">
-        <v>2.0</v>
-      </c>
-      <c r="E18" s="5">
+        <v>13</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D18" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="E18" s="3">
         <v>0.0</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2">
-        <v>46055.0</v>
+        <v>46046.0</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="C19" s="4" t="s">
-        <v>19</v>
+        <v>13</v>
+      </c>
+      <c r="C19" s="3" t="s">
+        <v>8</v>
       </c>
       <c r="D19" s="3">
-        <v>0.0</v>
-      </c>
-      <c r="E19" s="5">
-        <v>-1.5</v>
+        <v>3.0</v>
+      </c>
+      <c r="E19" s="3">
+        <v>0.0</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2">
-        <v>46085.0</v>
+        <v>46046.0</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="C20" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="D20" s="5">
-        <v>3.0</v>
-      </c>
-      <c r="E20" s="5">
+      <c r="C20" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="D20" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="E20" s="3">
         <v>0.0</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1">
       <c r="A21" s="2">
-        <v>46085.0</v>
+        <v>46046.0</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="C21" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="D21" s="5">
-        <v>2.0</v>
-      </c>
-      <c r="E21" s="5">
+        <v>13</v>
+      </c>
+      <c r="C21" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="D21" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="E21" s="3">
         <v>0.0</v>
       </c>
     </row>
     <row r="22" ht="15.75" customHeight="1">
       <c r="A22" s="2">
-        <v>46085.0</v>
+        <v>46046.0</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="C22" s="4" t="s">
-        <v>19</v>
+        <v>14</v>
+      </c>
+      <c r="C22" s="3" t="s">
+        <v>6</v>
       </c>
       <c r="D22" s="3">
-        <v>0.0</v>
-      </c>
-      <c r="E22" s="5">
-        <v>-1.5</v>
+        <v>3.0</v>
+      </c>
+      <c r="E22" s="3">
+        <v>0.0</v>
       </c>
     </row>
     <row r="23" ht="15.75" customHeight="1">
       <c r="A23" s="2">
-        <v>46117.0</v>
+        <v>46046.0</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="C23" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="D23" s="5">
-        <v>3.0</v>
-      </c>
-      <c r="E23" s="5">
+        <v>14</v>
+      </c>
+      <c r="C23" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D23" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="E23" s="3">
         <v>0.0</v>
       </c>
     </row>
     <row r="24" ht="15.75" customHeight="1">
       <c r="A24" s="2">
-        <v>46117.0</v>
+        <v>46046.0</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="C24" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="D24" s="5">
-        <v>2.0</v>
-      </c>
-      <c r="E24" s="5">
+        <v>14</v>
+      </c>
+      <c r="C24" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D24" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="E24" s="3">
         <v>0.0</v>
       </c>
     </row>
     <row r="25" ht="15.75" customHeight="1">
       <c r="A25" s="2">
-        <v>46117.0</v>
+        <v>46046.0</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="C25" s="4" t="s">
-        <v>13</v>
+        <v>14</v>
+      </c>
+      <c r="C25" s="3" t="s">
+        <v>9</v>
       </c>
       <c r="D25" s="3">
         <v>0.0</v>
       </c>
-      <c r="E25" s="5">
-        <v>-1.5</v>
+      <c r="E25" s="3">
+        <v>0.0</v>
       </c>
     </row>
     <row r="26" ht="15.75" customHeight="1">
       <c r="A26" s="2">
-        <v>46143.0</v>
+        <v>46046.0</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="C26" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="D26" s="5">
-        <v>3.0</v>
-      </c>
-      <c r="E26" s="5">
-        <v>0.0</v>
-      </c>
-    </row>
-    <row r="27" ht="15.75" customHeight="1">
-      <c r="A27" s="2">
-        <v>46143.0</v>
-      </c>
-      <c r="B27" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="C27" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="D27" s="5">
-        <v>2.0</v>
-      </c>
-      <c r="E27" s="5">
-        <v>0.0</v>
-      </c>
-    </row>
-    <row r="28" ht="15.75" customHeight="1">
-      <c r="A28" s="2">
-        <v>46143.0</v>
-      </c>
-      <c r="B28" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="C28" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="D28" s="3">
-        <v>0.0</v>
-      </c>
-      <c r="E28" s="5">
-        <v>-1.0</v>
-      </c>
-    </row>
-    <row r="29" ht="15.75" customHeight="1">
-      <c r="A29" s="2">
-        <v>46143.0</v>
-      </c>
-      <c r="B29" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="C29" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="D29" s="3">
-        <v>0.0</v>
-      </c>
-      <c r="E29" s="5">
-        <v>-1.5</v>
-      </c>
-    </row>
-    <row r="30" ht="15.75" customHeight="1">
-      <c r="A30" s="2">
-        <v>46203.0</v>
-      </c>
-      <c r="B30" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="C30" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="D30" s="3">
-        <v>2.0</v>
-      </c>
-      <c r="E30" s="3">
-        <v>0.0</v>
-      </c>
-    </row>
-    <row r="31" ht="15.75" customHeight="1">
-      <c r="A31" s="2">
-        <v>46203.0</v>
-      </c>
-      <c r="B31" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="C31" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="D31" s="3">
-        <v>0.0</v>
-      </c>
-      <c r="E31" s="3">
-        <v>0.0</v>
-      </c>
-    </row>
-    <row r="32" ht="15.75" customHeight="1">
-      <c r="A32" s="2">
-        <v>46203.0</v>
-      </c>
-      <c r="B32" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="C32" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="D32" s="3">
-        <v>0.0</v>
-      </c>
-      <c r="E32" s="3">
-        <v>-1.5</v>
-      </c>
-    </row>
-    <row r="33" ht="15.75" customHeight="1">
-      <c r="A33" s="2">
-        <v>46203.0</v>
-      </c>
-      <c r="B33" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="C33" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="D33" s="3">
-        <v>3.0</v>
-      </c>
-      <c r="E33" s="3">
-        <v>-1.0</v>
-      </c>
-    </row>
-    <row r="34" ht="15.75" customHeight="1">
-      <c r="A34" s="2">
-        <v>46203.0</v>
-      </c>
-      <c r="B34" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="C34" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="D34" s="3">
-        <v>0.0</v>
-      </c>
-      <c r="E34" s="3">
-        <v>0.0</v>
-      </c>
-    </row>
-    <row r="35" ht="15.75" customHeight="1">
-      <c r="A35" s="2">
-        <v>46218.0</v>
-      </c>
-      <c r="B35" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="C35" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="D35" s="3">
-        <v>3.0</v>
-      </c>
-      <c r="E35" s="3">
-        <v>0.0</v>
-      </c>
-    </row>
-    <row r="36" ht="15.75" customHeight="1">
-      <c r="A36" s="2">
-        <v>46218.0</v>
-      </c>
-      <c r="B36" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="C36" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="D36" s="3">
-        <v>2.0</v>
-      </c>
-      <c r="E36" s="3">
-        <v>0.0</v>
-      </c>
-    </row>
-    <row r="37" ht="15.75" customHeight="1">
-      <c r="A37" s="2">
-        <v>46218.0</v>
-      </c>
-      <c r="B37" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="C37" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D37" s="3">
-        <v>0.0</v>
-      </c>
-      <c r="E37" s="3">
-        <v>0.0</v>
-      </c>
-    </row>
-    <row r="38" ht="15.75" customHeight="1">
-      <c r="A38" s="2">
-        <v>46218.0</v>
-      </c>
-      <c r="B38" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="C38" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="D38" s="3">
-        <v>0.0</v>
-      </c>
-      <c r="E38" s="3">
-        <v>-1.0</v>
-      </c>
-    </row>
-    <row r="39" ht="15.75" customHeight="1">
-      <c r="A39" s="2">
-        <v>46218.0</v>
-      </c>
-      <c r="B39" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="C39" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="D39" s="3">
-        <v>0.0</v>
-      </c>
-      <c r="E39" s="3">
-        <v>-1.5</v>
-      </c>
-    </row>
-    <row r="40" ht="15.75" customHeight="1">
-      <c r="A40" s="2">
-        <v>46239.0</v>
-      </c>
-      <c r="B40" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="C40" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="D40" s="3">
-        <v>3.0</v>
-      </c>
-      <c r="E40" s="3">
-        <v>0.0</v>
-      </c>
-    </row>
-    <row r="41" ht="15.75" customHeight="1">
-      <c r="A41" s="2">
-        <v>46239.0</v>
-      </c>
-      <c r="B41" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="C41" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="D41" s="3">
-        <v>2.0</v>
-      </c>
-      <c r="E41" s="3">
-        <v>0.0</v>
-      </c>
-    </row>
-    <row r="42" ht="15.75" customHeight="1">
-      <c r="A42" s="2">
-        <v>46239.0</v>
-      </c>
-      <c r="B42" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="C42" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="D42" s="3">
-        <v>0.0</v>
-      </c>
-      <c r="E42" s="3">
-        <v>0.0</v>
-      </c>
-    </row>
-    <row r="43" ht="15.75" customHeight="1">
-      <c r="A43" s="2">
-        <v>46239.0</v>
-      </c>
-      <c r="B43" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="C43" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="D43" s="3">
-        <v>0.0</v>
-      </c>
-      <c r="E43" s="3">
-        <v>-1.0</v>
-      </c>
-    </row>
-    <row r="44" ht="15.75" customHeight="1">
-      <c r="A44" s="2">
-        <v>46239.0</v>
-      </c>
-      <c r="B44" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="C44" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="D44" s="3">
-        <v>0.0</v>
-      </c>
-      <c r="E44" s="3">
-        <v>-1.5</v>
-      </c>
-    </row>
-    <row r="45" ht="15.75" customHeight="1">
-      <c r="A45" s="6">
-        <v>46037.0</v>
-      </c>
-      <c r="B45" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="C45" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="D45" s="5">
-        <v>3.0</v>
-      </c>
-      <c r="E45" s="5">
-        <v>0.0</v>
-      </c>
-    </row>
-    <row r="46" ht="15.75" customHeight="1">
-      <c r="A46" s="6">
-        <v>46037.0</v>
-      </c>
-      <c r="B46" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="C46" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="D46" s="5">
-        <v>2.0</v>
-      </c>
-      <c r="E46" s="5">
-        <v>0.0</v>
-      </c>
-    </row>
-    <row r="47" ht="15.75" customHeight="1">
-      <c r="A47" s="6">
-        <v>46037.0</v>
-      </c>
-      <c r="B47" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="C47" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="D47" s="5">
-        <v>0.0</v>
-      </c>
-      <c r="E47" s="5">
-        <v>-1.0</v>
-      </c>
-    </row>
-    <row r="48" ht="15.75" customHeight="1">
-      <c r="A48" s="6">
-        <v>46037.0</v>
-      </c>
-      <c r="B48" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="C48" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="D48" s="5">
-        <v>0.0</v>
-      </c>
-      <c r="E48" s="5">
-        <v>-1.5</v>
-      </c>
-    </row>
-    <row r="49" ht="15.75" customHeight="1">
-      <c r="A49" s="6">
-        <v>46037.0</v>
-      </c>
-      <c r="B49" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="C49" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="D49" s="5">
-        <v>3.0</v>
-      </c>
-      <c r="E49" s="5">
-        <v>0.0</v>
-      </c>
-    </row>
-    <row r="50" ht="15.75" customHeight="1">
-      <c r="A50" s="6">
-        <v>46037.0</v>
-      </c>
-      <c r="B50" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="C50" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="D50" s="5">
-        <v>2.0</v>
-      </c>
-      <c r="E50" s="5">
-        <v>0.0</v>
-      </c>
-    </row>
-    <row r="51" ht="15.75" customHeight="1">
-      <c r="A51" s="6">
-        <v>46037.0</v>
-      </c>
-      <c r="B51" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="C51" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="D51" s="5">
-        <v>0.0</v>
-      </c>
-      <c r="E51" s="5">
-        <v>0.0</v>
-      </c>
-    </row>
-    <row r="52" ht="15.75" customHeight="1">
-      <c r="A52" s="6">
-        <v>46037.0</v>
-      </c>
-      <c r="B52" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="C52" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="D52" s="5">
-        <v>0.0</v>
-      </c>
-      <c r="E52" s="5">
-        <v>-1.0</v>
-      </c>
-    </row>
-    <row r="53" ht="15.75" customHeight="1">
-      <c r="A53" s="6">
-        <v>46037.0</v>
-      </c>
-      <c r="B53" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="C53" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="D53" s="5">
-        <v>0.0</v>
-      </c>
-      <c r="E53" s="5">
-        <v>-1.5</v>
-      </c>
-    </row>
+      <c r="C26" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="D26" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="E26" s="3">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="27" ht="15.75" customHeight="1"/>
+    <row r="28" ht="15.75" customHeight="1"/>
+    <row r="29" ht="15.75" customHeight="1"/>
+    <row r="30" ht="15.75" customHeight="1"/>
+    <row r="31" ht="15.75" customHeight="1"/>
+    <row r="32" ht="15.75" customHeight="1"/>
+    <row r="33" ht="15.75" customHeight="1"/>
+    <row r="34" ht="15.75" customHeight="1"/>
+    <row r="35" ht="15.75" customHeight="1"/>
+    <row r="36" ht="15.75" customHeight="1"/>
+    <row r="37" ht="15.75" customHeight="1"/>
+    <row r="38" ht="15.75" customHeight="1"/>
+    <row r="39" ht="15.75" customHeight="1"/>
+    <row r="40" ht="15.75" customHeight="1"/>
+    <row r="41" ht="15.75" customHeight="1"/>
+    <row r="42" ht="15.75" customHeight="1"/>
+    <row r="43" ht="15.75" customHeight="1"/>
+    <row r="44" ht="15.75" customHeight="1"/>
+    <row r="45" ht="15.75" customHeight="1"/>
+    <row r="46" ht="15.75" customHeight="1"/>
+    <row r="47" ht="15.75" customHeight="1"/>
+    <row r="48" ht="15.75" customHeight="1"/>
+    <row r="49" ht="15.75" customHeight="1"/>
+    <row r="50" ht="15.75" customHeight="1"/>
+    <row r="51" ht="15.75" customHeight="1"/>
+    <row r="52" ht="15.75" customHeight="1"/>
+    <row r="53" ht="15.75" customHeight="1"/>
     <row r="54" ht="15.75" customHeight="1"/>
     <row r="55" ht="15.75" customHeight="1"/>
     <row r="56" ht="15.75" customHeight="1"/>
@@ -2215,33 +1736,6 @@
     <row r="971" ht="15.75" customHeight="1"/>
     <row r="972" ht="15.75" customHeight="1"/>
     <row r="973" ht="15.75" customHeight="1"/>
-    <row r="974" ht="15.75" customHeight="1"/>
-    <row r="975" ht="15.75" customHeight="1"/>
-    <row r="976" ht="15.75" customHeight="1"/>
-    <row r="977" ht="15.75" customHeight="1"/>
-    <row r="978" ht="15.75" customHeight="1"/>
-    <row r="979" ht="15.75" customHeight="1"/>
-    <row r="980" ht="15.75" customHeight="1"/>
-    <row r="981" ht="15.75" customHeight="1"/>
-    <row r="982" ht="15.75" customHeight="1"/>
-    <row r="983" ht="15.75" customHeight="1"/>
-    <row r="984" ht="15.75" customHeight="1"/>
-    <row r="985" ht="15.75" customHeight="1"/>
-    <row r="986" ht="15.75" customHeight="1"/>
-    <row r="987" ht="15.75" customHeight="1"/>
-    <row r="988" ht="15.75" customHeight="1"/>
-    <row r="989" ht="15.75" customHeight="1"/>
-    <row r="990" ht="15.75" customHeight="1"/>
-    <row r="991" ht="15.75" customHeight="1"/>
-    <row r="992" ht="15.75" customHeight="1"/>
-    <row r="993" ht="15.75" customHeight="1"/>
-    <row r="994" ht="15.75" customHeight="1"/>
-    <row r="995" ht="15.75" customHeight="1"/>
-    <row r="996" ht="15.75" customHeight="1"/>
-    <row r="997" ht="15.75" customHeight="1"/>
-    <row r="998" ht="15.75" customHeight="1"/>
-    <row r="999" ht="15.75" customHeight="1"/>
-    <row r="1000" ht="15.75" customHeight="1"/>
   </sheetData>
   <printOptions/>
   <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>

</xml_diff>